<commit_message>
NAKO-2 DD and DPE for NAKO
</commit_message>
<xml_diff>
--- a/analyst/Ines/rmonize/data_dictionary/DD_NAKO_INES.xlsx
+++ b/analyst/Ines/rmonize/data_dictionary/DD_NAKO_INES.xlsx
@@ -1,22 +1,188 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\perrar\Documents\Perrar\NFDI4Health\TA5_1\use-cases-harmonisation\analyst\Ines\rmonize\data_dictionary\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="240" yWindow="20" windowWidth="16100" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Variables" sheetId="1" r:id="rId1"/>
     <sheet name="Categories" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="52">
+  <si>
+    <t>index</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>label</t>
+  </si>
+  <si>
+    <t>valueType</t>
+  </si>
+  <si>
+    <t>variable</t>
+  </si>
+  <si>
+    <t>sa_trig</t>
+  </si>
+  <si>
+    <t>sa_chol</t>
+  </si>
+  <si>
+    <t>sa_ldlc</t>
+  </si>
+  <si>
+    <t>sa_hdlc</t>
+  </si>
+  <si>
+    <t>a_anthro_bmi</t>
+  </si>
+  <si>
+    <t>anthro_bmi</t>
+  </si>
+  <si>
+    <t>anthro_hueftumfang</t>
+  </si>
+  <si>
+    <t>a_anthro_fettmasse</t>
+  </si>
+  <si>
+    <t>basis_age</t>
+  </si>
+  <si>
+    <t>GCAL</t>
+  </si>
+  <si>
+    <t>ZK</t>
+  </si>
+  <si>
+    <t>ZE</t>
+  </si>
+  <si>
+    <t>ZF</t>
+  </si>
+  <si>
+    <t>ZA</t>
+  </si>
+  <si>
+    <t>ZB</t>
+  </si>
+  <si>
+    <t>FS</t>
+  </si>
+  <si>
+    <t>FU</t>
+  </si>
+  <si>
+    <t>FP</t>
+  </si>
+  <si>
+    <t>KMD</t>
+  </si>
+  <si>
+    <t>KMT</t>
+  </si>
+  <si>
+    <t>KMF</t>
+  </si>
+  <si>
+    <t>MNA</t>
+  </si>
+  <si>
+    <t>MK</t>
+  </si>
+  <si>
+    <t>Triglyceride (trig): Messwert oder Fehlercode (6stellig)</t>
+  </si>
+  <si>
+    <t>Cholesterin, gesamt (chol): Messwert oder Fehlercode (6stellig)</t>
+  </si>
+  <si>
+    <t>LDL-Cholesterin (ldlc): Messwert oder Fehlercode (6stellig)</t>
+  </si>
+  <si>
+    <t>HDL-Cholesterin (hdlc): Messwert oder Fehlercode (6stellig)</t>
+  </si>
+  <si>
+    <t>decimal</t>
+  </si>
+  <si>
+    <t>BMI (aus bereinigten Messwerten)</t>
+  </si>
+  <si>
+    <t>BMI (at U2)</t>
+  </si>
+  <si>
+    <t>Hüftumfang</t>
+  </si>
+  <si>
+    <t>Bereinigter Körperfettanteil in % gemessen und automatisch oder manuell eingetragen</t>
+  </si>
+  <si>
+    <t>Alter am Untersuchungsdatum</t>
+  </si>
+  <si>
+    <t>Energie (Kilokalorien)  [kcal/d]</t>
+  </si>
+  <si>
+    <t>Kohlenhydrate, resorbierbar  [mg/d]</t>
+  </si>
+  <si>
+    <t>Eiweiß (Protein)  [mg/d]</t>
+  </si>
+  <si>
+    <t>Fett  [mg/d]</t>
+  </si>
+  <si>
+    <t>Ballaststoffe  [mg/d]</t>
+  </si>
+  <si>
+    <t>Gesättigte Fettsäuren  [mg/d]</t>
+  </si>
+  <si>
+    <t>Einfach ungesättigte Fettsäuren  [mg/d]</t>
+  </si>
+  <si>
+    <t>Mehrfach ungesättigte Fettsäuren  [mg/d]</t>
+  </si>
+  <si>
+    <t>Zucker (gesamt)  [mg/d]</t>
+  </si>
+  <si>
+    <t>Glucose (Traubenzucker)  [mg/d]</t>
+  </si>
+  <si>
+    <t>Fructose (Fruchtzucker)  [mg/d]</t>
+  </si>
+  <si>
+    <t>Natrium  [mg/d]</t>
+  </si>
+  <si>
+    <t>Alkohol (Ethanol)  [mg/d]</t>
+  </si>
+  <si>
+    <t>Kalium  [mg/d]</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -28,6 +194,39 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -50,25 +249,62 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  <cellStyles count="4">
+    <cellStyle name="Hyperlink" xfId="2"/>
+    <cellStyle name="Hyperlink 2" xfId="3"/>
+    <cellStyle name="Normal 2" xfId="1"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -110,7 +346,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -142,9 +378,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -176,6 +413,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -351,30 +589,279 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D24"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="25.6328125" customWidth="1"/>
+    <col min="3" max="3" width="33.81640625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>index</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>label</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>valueType</t>
-        </is>
+    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="B2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="B3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="B4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="58" x14ac:dyDescent="0.35">
+      <c r="B5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="B6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B7" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B8" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="B9" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="B10" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B11" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11" t="s">
+        <v>38</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B12" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C12" t="s">
+        <v>39</v>
+      </c>
+      <c r="D12" s="12" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B13" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" t="s">
+        <v>40</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B14" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C14" t="s">
+        <v>41</v>
+      </c>
+      <c r="D14" s="12" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B15" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="D15" s="12" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B16" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C16" t="s">
+        <v>42</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="17" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B17" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C17" t="s">
+        <v>43</v>
+      </c>
+      <c r="D17" s="12" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="18" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B18" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C18" t="s">
+        <v>44</v>
+      </c>
+      <c r="D18" s="12" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="19" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B19" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C19" t="s">
+        <v>45</v>
+      </c>
+      <c r="D19" s="12" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="20" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B20" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C20" t="s">
+        <v>46</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="21" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B21" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C21" t="s">
+        <v>47</v>
+      </c>
+      <c r="D21" s="12" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="22" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B22" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C22" t="s">
+        <v>48</v>
+      </c>
+      <c r="D22" s="12" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="23" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B23" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C23" t="s">
+        <v>49</v>
+      </c>
+      <c r="D23" s="12" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="24" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B24" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D24" s="12" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -383,25 +870,19 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>variable</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>label</t>
-        </is>
+    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
NAKO breakages removed from INES files. PREV_HYP: replaced with a_diab.
</commit_message>
<xml_diff>
--- a/analyst/Ines/rmonize/data_dictionary/DD_NAKO_INES.xlsx
+++ b/analyst/Ines/rmonize/data_dictionary/DD_NAKO_INES.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\use-cases-harmonisation\use-cases-harmonisation\analyst\Ines\rmonize\data_dictionary\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57D72E47-3F99-4C1E-89F7-BA63CDC7F3F7}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E84CC9BF-3DD5-4070-ACFC-2807E1F425F1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="13890" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -166,10 +166,6 @@
     <t>a_nu_kmt</t>
   </si>
   <si>
-    <t xml:space="preserve">
-a_nu_kmf</t>
-  </si>
-  <si>
     <t>Polysaccharide [mg/d]</t>
   </si>
   <si>
@@ -185,18 +181,19 @@
     <t>a_nu_zb</t>
   </si>
   <si>
-    <t xml:space="preserve">anthro_taillenumfang_fup
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">anthro_taillenumfang
-</t>
-  </si>
-  <si>
     <t>age_anth_fup</t>
   </si>
   <si>
     <t>gcal</t>
+  </si>
+  <si>
+    <t>anthro_taillenumfang</t>
+  </si>
+  <si>
+    <t>a_nu_kmf</t>
+  </si>
+  <si>
+    <t>anthro_taillenumfang_fup</t>
   </si>
 </sst>
 </file>
@@ -726,13 +723,13 @@
         <v>10</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D7" s="12" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:4" s="12" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B8" s="2" t="s">
         <v>53</v>
       </c>
@@ -743,9 +740,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:4" s="12" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B9" s="2" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C9" s="11" t="s">
         <v>43</v>
@@ -770,7 +767,7 @@
         <v>27</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D11" s="12" t="s">
         <v>13</v>
@@ -789,7 +786,7 @@
     </row>
     <row r="13" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="B13" s="3" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C13" s="11" t="s">
         <v>44</v>
@@ -800,7 +797,7 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B14" s="2" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C14" t="s">
         <v>16</v>
@@ -855,7 +852,7 @@
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B19" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C19" t="s">
         <v>20</v>
@@ -869,7 +866,7 @@
         <v>35</v>
       </c>
       <c r="C20" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D20" s="12" t="s">
         <v>13</v>
@@ -880,7 +877,7 @@
         <v>36</v>
       </c>
       <c r="C21" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D21" s="12" t="s">
         <v>13</v>
@@ -908,9 +905,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="24" spans="2:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B24" s="2" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="C24" t="s">
         <v>23</v>

</xml_diff>

<commit_message>
NAKO-5 changes to reflect NAKO dataset structure
</commit_message>
<xml_diff>
--- a/analyst/Ines/rmonize/data_dictionary/DD_NAKO_INES.xlsx
+++ b/analyst/Ines/rmonize/data_dictionary/DD_NAKO_INES.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\use-cases-harmonisation\use-cases-harmonisation\analyst\Ines\rmonize\data_dictionary\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\schwarz-f\Desktop\use-cases-harmonisation\analyst\Ines\rmonize\data_dictionary\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E84CC9BF-3DD5-4070-ACFC-2807E1F425F1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{748F7D00-A3BB-4784-8E54-FE351E553B9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="13890" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Variables" sheetId="1" r:id="rId1"/>
@@ -181,9 +181,6 @@
     <t>a_nu_zb</t>
   </si>
   <si>
-    <t>age_anth_fup</t>
-  </si>
-  <si>
     <t>gcal</t>
   </si>
   <si>
@@ -194,6 +191,9 @@
   </si>
   <si>
     <t>anthro_taillenumfang_fup</t>
+  </si>
+  <si>
+    <t>basis_age_fup</t>
   </si>
 </sst>
 </file>
@@ -305,8 +305,8 @@
   <cellStyles count="4">
     <cellStyle name="Hyperlink" xfId="2" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
     <cellStyle name="Hyperlink 2" xfId="3" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -322,9 +322,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -362,9 +362,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -397,26 +397,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -449,26 +432,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -643,7 +609,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D27"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="25.5703125" customWidth="1"/>
     <col min="3" max="3" width="33.85546875" customWidth="1"/>
@@ -731,7 +697,7 @@
     </row>
     <row r="8" spans="1:4" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B8" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C8" s="11" t="s">
         <v>41</v>
@@ -742,7 +708,7 @@
     </row>
     <row r="9" spans="1:4" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B9" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C9" s="11" t="s">
         <v>43</v>
@@ -786,7 +752,7 @@
     </row>
     <row r="13" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="B13" s="3" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C13" s="11" t="s">
         <v>44</v>
@@ -797,7 +763,7 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B14" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C14" t="s">
         <v>16</v>
@@ -907,7 +873,7 @@
     </row>
     <row r="24" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B24" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C24" t="s">
         <v>23</v>
@@ -949,7 +915,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C1"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">

</xml_diff>

<commit_message>
NAKO-5, changes to ines document names
</commit_message>
<xml_diff>
--- a/analyst/Ines/rmonize/data_dictionary/DD_NAKO_INES.xlsx
+++ b/analyst/Ines/rmonize/data_dictionary/DD_NAKO_INES.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\schwarz-f\Desktop\use-cases-harmonisation\analyst\Ines\rmonize\data_dictionary\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{748F7D00-A3BB-4784-8E54-FE351E553B9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CACF3693-17DC-41C0-A3F5-9674036BCF69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Variables" sheetId="1" r:id="rId1"/>
@@ -58,9 +58,6 @@
     <t>a_anthro_bmi</t>
   </si>
   <si>
-    <t>anthro_bmi</t>
-  </si>
-  <si>
     <t>anthro_hueftumfang</t>
   </si>
   <si>
@@ -181,9 +178,6 @@
     <t>a_nu_zb</t>
   </si>
   <si>
-    <t>gcal</t>
-  </si>
-  <si>
     <t>anthro_taillenumfang</t>
   </si>
   <si>
@@ -194,6 +188,12 @@
   </si>
   <si>
     <t>basis_age_fup</t>
+  </si>
+  <si>
+    <t>anthro_BMI</t>
+  </si>
+  <si>
+    <t>a_nu_gcal</t>
   </si>
 </sst>
 </file>
@@ -634,10 +634,10 @@
         <v>5</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -645,10 +645,10 @@
         <v>6</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -656,10 +656,10 @@
         <v>7</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -667,10 +667,10 @@
         <v>8</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -678,230 +678,230 @@
         <v>9</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B7" s="4" t="s">
-        <v>10</v>
+        <v>54</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:4" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B8" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:4" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B9" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B10" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="11" spans="1:4" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B11" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="B12" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="B13" s="3" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D13" s="12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B14" s="2" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D14" s="12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B15" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C15" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D15" s="12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B16" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C16" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D16" s="12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B17" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C17" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B18" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B19" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C19" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B20" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C20" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B21" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C21" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="22" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B22" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C22" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="23" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B23" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C23" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D23" s="12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="24" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B24" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C24" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="25" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B25" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C25" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D25" s="12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="26" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B26" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D26" s="12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="27" spans="2:4" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
NAKO-5: including special numbers for missingness in the files
</commit_message>
<xml_diff>
--- a/analyst/Ines/rmonize/data_dictionary/DD_NAKO_INES.xlsx
+++ b/analyst/Ines/rmonize/data_dictionary/DD_NAKO_INES.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\schwarz-f\Desktop\use-cases-harmonisation\analyst\Ines\rmonize\data_dictionary\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CACF3693-17DC-41C0-A3F5-9674036BCF69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7BFED4C-A6E4-4306-9852-40CD087D2178}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Variables" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="74">
   <si>
     <t>index</t>
   </si>
@@ -194,6 +194,60 @@
   </si>
   <si>
     <t>a_nu_gcal</t>
+  </si>
+  <si>
+    <t>missing</t>
+  </si>
+  <si>
+    <t>TRUE</t>
+  </si>
+  <si>
+    <t>Sample too old</t>
+  </si>
+  <si>
+    <t>Hemolytic sample</t>
+  </si>
+  <si>
+    <t>lipemic sample</t>
+  </si>
+  <si>
+    <t>Technically not possible</t>
+  </si>
+  <si>
+    <t>Planned not determined</t>
+  </si>
+  <si>
+    <t>no valid information available</t>
+  </si>
+  <si>
+    <t>Eliminated by group of experts</t>
+  </si>
+  <si>
+    <t>missing due to impossible calculation</t>
+  </si>
+  <si>
+    <t>Implausible information</t>
+  </si>
+  <si>
+    <t>Calculation not possible due to implausible values</t>
+  </si>
+  <si>
+    <t>Allowed skipped</t>
+  </si>
+  <si>
+    <t>Not specified</t>
+  </si>
+  <si>
+    <t>Don't know</t>
+  </si>
+  <si>
+    <t>Not specified, erroneously skipped</t>
+  </si>
+  <si>
+    <t>missing data</t>
+  </si>
+  <si>
+    <t>calculation not possible due to implausible</t>
   </si>
 </sst>
 </file>
@@ -273,7 +327,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -301,6 +355,8 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Hyperlink" xfId="2" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -914,10 +970,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="24.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="79.140625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -926,6 +987,541 @@
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="12">
+        <v>111111</v>
+      </c>
+      <c r="C2" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="D2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="12">
+        <v>222222</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="12">
+        <v>333333</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="12">
+        <v>444444</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="12">
+        <v>555555</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="12">
+        <v>999999</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" s="12">
+        <v>111111</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" s="12">
+        <v>222222</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10" s="12">
+        <v>333333</v>
+      </c>
+      <c r="C10" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="B11" s="12">
+        <v>444444</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="B12" s="12">
+        <v>555555</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="D12" s="12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="B13" s="12">
+        <v>999999</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="B14" s="12">
+        <v>666666</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="D14" s="12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="B15" s="12">
+        <v>111111</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="D15" s="12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="B16" s="12">
+        <v>222222</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="B17" s="12">
+        <v>333333</v>
+      </c>
+      <c r="C17" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="D17" s="12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="B18" s="12">
+        <v>444444</v>
+      </c>
+      <c r="C18" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="D18" s="12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="B19" s="12">
+        <v>555555</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="D19" s="12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="B20" s="12">
+        <v>999999</v>
+      </c>
+      <c r="C20" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="B21" s="12">
+        <v>666666</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="D21" s="12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B22" s="12">
+        <v>7777</v>
+      </c>
+      <c r="C22" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="D22" s="12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B23" s="12">
+        <v>8886</v>
+      </c>
+      <c r="C23" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="D23" s="12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B24" s="12">
+        <v>7776</v>
+      </c>
+      <c r="C24" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="D24" s="12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B25" s="12">
+        <v>7775</v>
+      </c>
+      <c r="C25" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="D25" s="12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B26" s="12">
+        <v>8888</v>
+      </c>
+      <c r="C26" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="D26" s="12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B27" s="12">
+        <v>9999</v>
+      </c>
+      <c r="C27" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="D27" s="12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B28" s="12">
+        <v>8889</v>
+      </c>
+      <c r="C28" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="D28" s="12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B29" s="12">
+        <v>7777</v>
+      </c>
+      <c r="C29" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="D29" s="12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B30" s="12">
+        <v>8886</v>
+      </c>
+      <c r="C30" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="D30" s="12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B31" s="12">
+        <v>7776</v>
+      </c>
+      <c r="C31" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="D31" s="12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B32" s="12">
+        <v>7775</v>
+      </c>
+      <c r="C32" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="D32" s="12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B33" s="12">
+        <v>8888</v>
+      </c>
+      <c r="C33" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="D33" s="12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B34" s="12">
+        <v>9999</v>
+      </c>
+      <c r="C34" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="D34" s="12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B35" s="12">
+        <v>8889</v>
+      </c>
+      <c r="C35" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="D35" s="12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B36" s="12">
+        <v>9999</v>
+      </c>
+      <c r="C36" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="D36" s="12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="B37" s="12">
+        <v>9999</v>
+      </c>
+      <c r="C37" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="D37" s="12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B38" s="12">
+        <v>9999</v>
+      </c>
+      <c r="C38" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="D38" s="12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B39" s="12">
+        <v>9999</v>
+      </c>
+      <c r="C39" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="D39" s="12" t="s">
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>